<commit_message>
Complete Final Clue 5-Path ODK package: update paths 1-5 with strict uppercase, mandatory constraints, updated riddles, image assets, and master keys
</commit_message>
<xml_diff>
--- a/ROUTE_1_PATH1_ECE_MECH_FC_CY_AUDI/PATH1_ANSWER_KEY.xlsx
+++ b/ROUTE_1_PATH1_ECE_MECH_FC_CY_AUDI/PATH1_ANSWER_KEY.xlsx
@@ -433,22 +433,22 @@
         <v>Start Desk</v>
       </c>
       <c r="C2" t="str">
-        <v>Team Setup</v>
+        <v>Team Setup &amp; Instructions</v>
       </c>
       <c r="D2" t="str">
-        <v>Enter Team ID &amp; Team Leader Name</v>
+        <v>Rules, Qualification Rules, Team ID &amp; Leader Name</v>
       </c>
       <c r="E2" t="str">
         <v>None</v>
       </c>
       <c r="F2" t="str">
-        <v>TEAM-XX (CAPS)</v>
+        <v>TEAM-XX (UPPERCASE ONLY)</v>
       </c>
       <c r="G2" t="str">
         <v>Strict UPPERCASE regex(., '^[A-Z0-9\-_ ]+$')</v>
       </c>
       <c r="H2" t="str">
-        <v>No</v>
+        <v>No (Input Mandatory)</v>
       </c>
     </row>
     <row r="3">
@@ -456,25 +456,25 @@
         <v>Round 1 (R1)</v>
       </c>
       <c r="B3" t="str">
-        <v>ECE Block</v>
+        <v>Starting Block (ECE)</v>
       </c>
       <c r="C3" t="str">
-        <v>🧩 Object Finding (Hidden Object)</v>
+        <v>Object Finding</v>
       </c>
       <c r="D3" t="str">
-        <v>Find assigned hidden object, take photo, enter volunteer code</v>
+        <v>Find assigned hidden object, upload photo, enter volunteer code</v>
       </c>
       <c r="E3" t="str">
         <v>None</v>
       </c>
       <c r="F3" t="str">
-        <v>R1-P1EC</v>
+        <v>R1-P1EC (UPPERCASE ONLY)</v>
       </c>
       <c r="G3" t="str">
-        <v>translate(...) = 'R1-P1EC'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'R1-P1EC'</v>
       </c>
       <c r="H3" t="str">
-        <v>Yes (Discovered Hidden Object Photo)</v>
+        <v>Yes (Discovered Hidden Object Photo — MANDATORY)</v>
       </c>
     </row>
     <row r="4">
@@ -485,74 +485,74 @@
         <v>In-App Audio Clue</v>
       </c>
       <c r="C4" t="str">
-        <v>Engine Sound Challenge</v>
+        <v>Audio Clue (No challenge name displayed)</v>
       </c>
       <c r="D4" t="str">
-        <v>Listen to engine_sound.mpeg, identify destination block &amp; enter arrival code</v>
+        <v>Listen to sound, identify academic block (MECH) &amp; enter start code</v>
       </c>
       <c r="E4" t="str">
         <v>engine_sound.mpeg</v>
       </c>
       <c r="F4" t="str">
-        <v>MECH (Destination) &amp; SOUND-PASS (Arrival Code)</v>
+        <v>MECH (or MECHANICAL BLOCK / MECH BLOCK) &amp; SOUND-PASS (UPPERCASE ONLY)</v>
       </c>
       <c r="G4" t="str">
-        <v>translate(...) = 'MECH' &amp; translate(...) = 'SOUND-PASS'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'MECH' &amp; 'SOUND-PASS'</v>
       </c>
       <c r="H4" t="str">
-        <v>No</v>
+        <v>No (Input Mandatory)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Round 2 (R2 Var 1)</v>
+        <v>Round 2 (R2 Var A)</v>
       </c>
       <c r="B5" t="str">
         <v>MECH Block</v>
       </c>
       <c r="C5" t="str">
-        <v>Human Shape Pose Challenge</v>
+        <v>Variant A: Human Poses</v>
       </c>
       <c r="D5" t="str">
-        <v>Recreate poses from volunteer poses page with 4 members, upload 4 mandatory photos, enter code</v>
+        <v>Perform any 4 poses shown by volunteer, upload 4 mandatory photos one by one, enter code</v>
       </c>
       <c r="E5" t="str">
-        <v>Poses page provided by volunteers</v>
+        <v>Poses shown by volunteers</v>
       </c>
       <c r="F5" t="str">
-        <v>MECH-PS-1</v>
+        <v>MECH-PS-1 (UPPERCASE ONLY)</v>
       </c>
       <c r="G5" t="str">
-        <v>translate(...) = 'MECH-PS-1'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'MECH-PS-1'</v>
       </c>
       <c r="H5" t="str">
-        <v>Yes (4 Mandatory Member Pose Photos)</v>
+        <v>Yes (4 Mandatory Photos of Poses — MANDATORY)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Round 2 (R2 Var 2)</v>
+        <v>Round 2 (R2 Var B)</v>
       </c>
       <c r="B6" t="str">
         <v>MECH Block</v>
       </c>
       <c r="C6" t="str">
-        <v>Paper Ball Challenge</v>
+        <v>Variant B: Paper Ball</v>
       </c>
       <c r="D6" t="str">
-        <v>Complete paper ball &amp; exam pads challenge, enter code</v>
+        <v>Complete challenge explained by volunteer, enter completion code</v>
       </c>
       <c r="E6" t="str">
         <v>None</v>
       </c>
       <c r="F6" t="str">
-        <v>ME-PB-1</v>
+        <v>ME-PB-1 (UPPERCASE ONLY)</v>
       </c>
       <c r="G6" t="str">
-        <v>translate(...) = 'ME-PB-1'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'ME-PB-1'</v>
       </c>
       <c r="H6" t="str">
-        <v>No</v>
+        <v>No (Input Mandatory)</v>
       </c>
     </row>
     <row r="7">
@@ -563,48 +563,48 @@
         <v>In-App Cipher</v>
       </c>
       <c r="C7" t="str">
-        <v>Shuffled Numbers</v>
+        <v>Shuffled Numbers (Displayed as ROUND 3)</v>
       </c>
       <c r="D7" t="str">
-        <v>Decode 11-4-15-7-12-21-4-16, 5-21-4-10-14, 5-18-23-23-15-8, 20-24-8-24-8, 6-18-24-17-23-8-21</v>
+        <v>Decode 5 words in separate slides: 11-4-15-7-12-21-4-16, 5-21-4-10-14, 5-18-23-23-15-8, 20-24-8-24-8, 6-18-24-17-23-8-21 -&gt; Destination guess</v>
       </c>
       <c r="E7" t="str">
         <v>None</v>
       </c>
       <c r="F7" t="str">
-        <v>HALDIRAM, BREAK, BOTTLE, QUEUE, COUNTER -&gt; Destination: FOOD COURT</v>
+        <v>HALDIRAM, BREAK, BOTTLE, QUEUE, COUNTER -&gt; Destination: FOOD COURT / FOOD CANTEEN / CANTEEN (UPPERCASE ONLY)</v>
       </c>
       <c r="G7" t="str">
-        <v>translate(...) on all 5 decoded words + FOOD COURT</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) on all 5 decoded words + FOOD COURT / FOOD CANTEEN / CANTEEN</v>
       </c>
       <c r="H7" t="str">
-        <v>No</v>
+        <v>No (All 6 Inputs MANDATORY)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Round 3 (R3)</v>
+        <v>Round 3 Checkpoint (R3)</v>
       </c>
       <c r="B8" t="str">
         <v>Food Court</v>
       </c>
       <c r="C8" t="str">
-        <v>QR Hunt</v>
+        <v>QR Hunt &amp; Volunteer Code</v>
       </c>
       <c r="D8" t="str">
-        <v>Find hidden QR code, scan with in-app barcode scanner</v>
+        <v>Find hidden QR code in a fun way, scan barcode scanner, enter volunteer completion code</v>
       </c>
       <c r="E8" t="str">
         <v>None</v>
       </c>
       <c r="F8" t="str">
-        <v>FAKE-ME-CYBER</v>
+        <v>Barcode: FAKE-ME-CYBER &amp; Code: QR-HUNT-GOOD (UPPERCASE ONLY)</v>
       </c>
       <c r="G8" t="str">
-        <v>Scanned value = 'FAKE-ME-CYBER'</v>
+        <v>Scanned value = 'FAKE-ME-CYBER' &amp; normalize-space(.) = 'QR-HUNT-GOOD'</v>
       </c>
       <c r="H8" t="str">
-        <v>No (Barcode Scanner)</v>
+        <v>Yes (Barcode Scan MANDATORY)</v>
       </c>
     </row>
     <row r="9">
@@ -624,39 +624,39 @@
         <v>None</v>
       </c>
       <c r="F9" t="str">
-        <v>CYBER (or CY / CY SEMINAR HALL / CYBER SEMINAR HALL)</v>
+        <v>CYBER (or CYBER SECURITY / CY / CY SEMINAR HALL) (UPPERCASE ONLY)</v>
       </c>
       <c r="G9" t="str">
-        <v>translate(...) = 'CYBER' / 'CY' / 'CY SEMINAR HALL'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'CYBER' / 'CYBER SECURITY' / 'CY'</v>
       </c>
       <c r="H9" t="str">
-        <v>No</v>
+        <v>No (Input Mandatory)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Round 4 (R4)</v>
+        <v>Round 4 Checkpoint (R4)</v>
       </c>
       <c r="B10" t="str">
         <v>CY Seminar Hall</v>
       </c>
       <c r="C10" t="str">
-        <v>Physical Agility Challenge</v>
+        <v>Physical Challenge &amp; Hall Navigation</v>
       </c>
       <c r="D10" t="str">
-        <v>Complete physical challenge with volunteers, enter code</v>
+        <v>Navigate hall, enter start code START-PHY, perform physical challenge, enter finish code PHY-CY</v>
       </c>
       <c r="E10" t="str">
         <v>None</v>
       </c>
       <c r="F10" t="str">
-        <v>PHY-CY</v>
+        <v>Start Code: START-PHY &amp; Finish Code: PHY-CY (UPPERCASE ONLY)</v>
       </c>
       <c r="G10" t="str">
-        <v>translate(...) = 'PHY-CY'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'START-PHY' &amp; 'PHY-CY'</v>
       </c>
       <c r="H10" t="str">
-        <v>No</v>
+        <v>No (Inputs Mandatory)</v>
       </c>
     </row>
     <row r="11">
@@ -676,13 +676,13 @@
         <v>None</v>
       </c>
       <c r="F11" t="str">
-        <v>AUDITORIUM (or AUDI)</v>
+        <v>AUDITORIUM (or AUDI) (UPPERCASE ONLY)</v>
       </c>
       <c r="G11" t="str">
-        <v>translate(...) = 'AUDITORIUM' or 'AUDI'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'AUDITORIUM' or 'AUDI'</v>
       </c>
       <c r="H11" t="str">
-        <v>No</v>
+        <v>No (Input Mandatory)</v>
       </c>
     </row>
     <row r="12">
@@ -702,39 +702,39 @@
         <v>None</v>
       </c>
       <c r="F12" t="str">
-        <v>STAGE</v>
+        <v>STAGE (UPPERCASE ONLY)</v>
       </c>
       <c r="G12" t="str">
-        <v>translate(...) = 'STAGE'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'STAGE'</v>
       </c>
       <c r="H12" t="str">
-        <v>No</v>
+        <v>No (Input Mandatory)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Final Completion</v>
+        <v>Grand Finale</v>
       </c>
       <c r="B13" t="str">
         <v>Main Auditorium Stage</v>
       </c>
       <c r="C13" t="str">
-        <v>Grand Finale Puzzle Verification</v>
+        <v>Tied Legs/Hands Rush, Solved Puzzle &amp; Bell Ring</v>
       </c>
       <c r="D13" t="str">
-        <v>Upload photo of solved puzzle &amp; enter chief judge clearance code</v>
+        <v>Go with legs &amp; hands tied, solve puzzle, upload photo of solved puzzle, enter clearance code FINAL-PATH1, run to ring the bell to win</v>
       </c>
       <c r="E13" t="str">
         <v>None</v>
       </c>
       <c r="F13" t="str">
-        <v>FINAL-PATH1</v>
+        <v>FINAL-PATH1 (UPPERCASE ONLY) -&gt; Ring Bell</v>
       </c>
       <c r="G13" t="str">
-        <v>translate(...) = 'FINAL-PATH1'</v>
+        <v>Strict UPPERCASE regex &amp; normalize-space(.) = 'FINAL-PATH1'</v>
       </c>
       <c r="H13" t="str">
-        <v>Yes (Solved Puzzle Photo)</v>
+        <v>Yes (Solved Puzzle Photo MANDATORY)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>